<commit_message>
Add AAAI and improve table layout
</commit_message>
<xml_diff>
--- a/data/core_conferences_normalized_tags.xlsx
+++ b/data/core_conferences_normalized_tags.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="R254c1bf86c46446c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="R5b88de0a90bf48c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core Conferences" sheetId="1" r:id="R9df255e54181423f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Vocabulary" sheetId="2" r:id="R4f20a8483e5f45ac"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -157,9 +157,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -951,10 +951,30 @@
         <x:v>https://chi2026.acm.org/</x:v>
       </x:c>
     </x:row>
+    <x:row r="35">
+      <x:c r="A35" t="str">
+        <x:v>AAAI</x:v>
+      </x:c>
+      <x:c r="B35" t="str">
+        <x:v>Machine Learning; Deep Representation Learning; Data Mining &amp; Data Science; Fairness &amp; Responsible AI</x:v>
+      </x:c>
+      <x:c r="C35" t="str">
+        <x:v>XXL</x:v>
+      </x:c>
+      <x:c r="D35" t="str">
+        <x:v>Very hard</x:v>
+      </x:c>
+      <x:c r="E35" t="str">
+        <x:v>Paper-based / OpenReview</x:v>
+      </x:c>
+      <x:c r="F35" t="str">
+        <x:v>https://aaai.org/conference/aaai/aaai-27/</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c5b258f0f5a4961"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c242cb4471d40d3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1106,7 +1126,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa6ae67cc45c4044"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5322ae3c56cb4fec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>